<commit_message>
feat: embed official Shulex customer service QR code across all READMEs and directly inside the Excel template
</commit_message>
<xml_diff>
--- a/projects/01-atomic-knowledge-base/excel/shulex_atomic_kb_template.xlsx
+++ b/projects/01-atomic-knowledge-base/excel/shulex_atomic_kb_template.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,12 @@
     <font>
       <name val="Microsoft YaHei"/>
       <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -99,15 +105,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,6 +197,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="1809750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -481,11 +518,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -626,6 +664,11 @@
           <t>清理下架产品与已作废的促销活动文档，保持知识库常新。</t>
         </is>
       </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>▲ 微信扫码添加 Shulex 官方顾问</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -638,9 +681,15 @@
           <t>导入 Shulex 智能客服系统，点击一键同步生效。</t>
         </is>
       </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>获取 1 对 1 知识库诊断与数字员工免费试用</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -663,7 +712,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>📋 表 1：全店基础政策与红线规矩表（底线问题 · 杜绝两头扯皮）</t>
         </is>
@@ -671,192 +720,192 @@
     </row>
     <row r="2"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>业务场景</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>触发条件</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>运费承担方</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>标准执行口径（无歧义结论）</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>例外或特殊说明</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>建议话术闭环动作</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>7天无理由退货</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>签收7天内，商品及配件齐全且不影响二次销售</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>买家承担（如有运费险由保司赔付）</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>支持7天无理由退换，寄回需确保原包装与配件完好。</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>贴身衣物/定制类拆封不退</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>发送退货地址与注意事项</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>商品质量问题/破损</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>签收48小时内提供破损照片或视频凭据</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>卖家全额承担</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>核实无误后免费补发或全额退款，运费由我方承担。</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>人为摔损或使用不当除外</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>引导上传照片并极速发起补发工单</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>发货时效与催单</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>付款后48小时内（大促预售除外）</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>不涉及</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>日常订单48小时内发货，顺丰/中通极速发出。</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>预售商品以商详标明发货时间为准</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>查询实时物流节点并同步给买家</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>发票开具</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>订单确认收货后</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>不涉及</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>支持开具电子增值税普通发票，确认收货后1-3个工作日开出。</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>专票需提供完整三证资质</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>发送开票信息登记快捷表单</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>质保与延保</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>自签收之日起1年内（核心配件2年）</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>前3个月卖家承担，后续双方各半</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>整机质保1年，非人为质量故障免费寄修或以换代修。</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>易损耗件（如滤网/电池）质保6个月</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>登记序列号并生成售后维修工单</t>
         </is>
@@ -889,7 +938,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>📐 表 2：产品与参数原子结构表（事实真理 · 杜绝 AI 参数幻觉）</t>
         </is>
@@ -897,128 +946,128 @@
     </row>
     <row r="2"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>商品名称/型号</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>核心参数（尺寸/电压/功率）</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>官方适配/兼容清单</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>明确不兼容清单</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>常见故障代码</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>对应排除方法与标准答复</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Shulex Pro 智能无线耳机</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>重量4.2g/单耳；续航32h；蓝牙5.3；Type-C 5V/1A</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>iOS 12+，Android 8+，Windows 10/11</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>不支持旧款蓝牙4.0及以下设备</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>红白灯交替慢闪</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>双耳放入充电盒长按底座按键10秒重置连接。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>桌面高速充电坞 65W</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>输入100-240V；氮化镓；GaN 65W Max；3C1A</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>PD3.0/QC4+/PPS协议笔记本/手机/平板</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>不支持非标直流设备、大功率电饭煲</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>白灯快闪2次后熄灭</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>过载保护触发，请拔掉超负荷设备等待30秒自动恢复。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>智能感应静音加湿器</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>水箱容量4.5L；额定功率25W；加湿量350ml/h</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>纯净水、凉开水</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>切勿直接加自来水、高浓度精油</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>缺水红灯常亮</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>水箱浮子卡住或水量不足，请清洁水箱并重新加水。</t>
         </is>
@@ -1051,7 +1100,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>💬 表 3：买家大白话与口语同义句表（桥接自然语言 · 杜绝答非所问）</t>
         </is>
@@ -1059,160 +1108,160 @@
     </row>
     <row r="2"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>标准业务问题</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>买家真实口语表达 (同义句1)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>买家真实口语表达 (同义句2)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>买家真实口语表达 (同义句3)</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>买家真实口语表达 (同义句4)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>AI 标准理解与答复重点</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>设备无法开机</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>按开关没反应</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>灯怎么都不亮</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>充了半天电还是死机</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>是不是坏了开不开</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>判断是否处于运输锁止状态或电量耗尽，给出长按5秒解锁指示。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>催物流/不更新</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>怎么三天了还没动静</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>快递卡在半路了吗</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>到底发没发货啊急死我了</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>今天能送到吗</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>安抚情绪并调取最新中转网点，超时主动启动丢件拦截补偿。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>申请换货运费补贴</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>寄回去运费谁出</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>运费怎么返还给我</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>先垫付的邮费怎么报销</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>你们承担运费吗</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>告知填写寄回单号后，系统将在签收次日自动原路返还至账户。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>颜色/尺寸不合心意</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>跟图片色差太大了吧</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>太小了根本装不下</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>感觉实物有点塑料感</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>买错型号了</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>共情审美差异，告知支持无理由极速调换对应尺码/色系。</t>
         </is>
@@ -1245,7 +1294,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>⚡ 表 4：决策与行动指令表（不只当复读机 · 真正闭环办事）</t>
         </is>
@@ -1253,128 +1302,128 @@
     </row>
     <row r="2"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>用户意图</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>触发前置条件</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>AI 判定等级</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>必须索要的信息</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>联动后台动作 (Action)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>闭环完成话术</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>配件漏发/破损补发</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>客户提供包裹面单 + 破损部件照片</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>L1 自动化</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>快递运单号、破损照片、收件地址确认</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>自动生成 ERP 补发工单，推送仓库排单</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>“已为您极速登记补发，单号将在发货后通过短信同步给您！”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>极速小额补偿</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>轻微瑕疵/物流延误且客户意向保留</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>L1 权限内(≤10元)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>支付宝账号或原路返还确认</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>触发店铺小额赔付接口，自动登记报销</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>“非常抱歉给您带来不便，小额补偿已为您极速退回原支付账户！”</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>大额投诉/疑难退换</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>多次沟通未果/提及工商投诉/差评</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>L2 转人工二线</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>联系电话、争议核心诉求</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>即时@值班客服主管钉钉/企微，附带完整对话摘要</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>“已为您升级资深服务专家跟进，我们将在 15 分钟内电话联系您！”</t>
         </is>

</xml_diff>